<commit_message>
Add GitHub Actions CI workflow, deployment configs, and deploy buttons
</commit_message>
<xml_diff>
--- a/public/exports/portfolio_database_export.xlsx
+++ b/public/exports/portfolio_database_export.xlsx
@@ -420,7 +420,7 @@
         <v>Full Name</v>
       </c>
       <c r="B2" t="str">
-        <v>Alex Vance Morgan</v>
+        <v>Pranav Santhosh Nair</v>
       </c>
     </row>
     <row r="3">
@@ -436,7 +436,7 @@
         <v>Email</v>
       </c>
       <c r="B4" t="str">
-        <v>alex.morgan.portfolio@example.com</v>
+        <v>2025.pranavs@isu.ac.in</v>
       </c>
     </row>
     <row r="5">
@@ -444,7 +444,7 @@
         <v>Phone</v>
       </c>
       <c r="B5" t="str">
-        <v>+1 (555) 382-9104</v>
+        <v>09920486737</v>
       </c>
     </row>
     <row r="6">
@@ -452,7 +452,7 @@
         <v>Location</v>
       </c>
       <c r="B6" t="str">
-        <v>San Francisco, CA (Open to Remote)</v>
+        <v xml:space="preserve">Kharghar </v>
       </c>
     </row>
     <row r="7">
@@ -460,7 +460,7 @@
         <v>LinkedIn</v>
       </c>
       <c r="B7" t="str">
-        <v>https://linkedin.com/in/alex-morgan-ai</v>
+        <v>https://linkedin.com/in/Prana_nair</v>
       </c>
     </row>
     <row r="8">
@@ -468,7 +468,7 @@
         <v>GitHub</v>
       </c>
       <c r="B8" t="str">
-        <v>https://github.com/alexmorgan-ai</v>
+        <v>https://github.com/PranavNair2007</v>
       </c>
     </row>
     <row r="9">
@@ -476,15 +476,18 @@
         <v>Portfolio URL</v>
       </c>
       <c r="B9" t="str">
-        <v>https://alexmorgan.dev</v>
-      </c>
-    </row>
-    <row r="10">
+        <v/>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
       <c r="A10" t="str">
         <v>Summary</v>
       </c>
-      <c r="B10" t="str">
-        <v>Versatile Senior Engineer with 6+ years of experience architecting high-scale distributed systems, enterprise full-stack applications, and production generative AI solutions. Proven record of deploying RAG architectures, multi-agent frameworks, and resilient cloud services serving millions of requests daily.</v>
+      <c r="B10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Languages: • 🐍 Python • 🌐 Basic HTML
+Tools: • 🧩 VS Code • 🧭 Git &amp; GitHub • 🤖 AI Google Studio
+Skills: • 🌐 Basic Web Development • 🔍 Problem Solving • 🧠 Logic Building
+</v>
       </c>
     </row>
     <row r="11">
@@ -492,7 +495,7 @@
         <v>Exported At</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-10-28T15:31:37.304Z</v>
+        <v>2026-10-28T16:14:58.769Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>